<commit_message>
Add links for main branch asset lists to asset list, readme
Add links for main branch asset lists to asset list, readme
</commit_message>
<xml_diff>
--- a/Asset Lists & Artifact Lists/artifact-list.xlsx
+++ b/Asset Lists & Artifact Lists/artifact-list.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mathewthomson/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mathewthomson/Documents/GitHub/.github/Asset Lists &amp; Artifact Lists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{1EE6371F-C331-DE4D-809A-F49E478A09F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD567381-FCB4-734A-A0FE-C5E182394CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1800" yWindow="1020" windowWidth="27240" windowHeight="16440" xr2:uid="{FB3463DD-60E6-9047-9A81-48DD9E965D16}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="249">
   <si>
     <t>assetID</t>
   </si>
@@ -579,18 +578,9 @@
     <t>18/12/2025</t>
   </si>
   <si>
-    <t>PHES-ODM Project Artifact List</t>
-  </si>
-  <si>
-    <t>odmArtifacts</t>
-  </si>
-  <si>
     <t>xlsx</t>
   </si>
   <si>
-    <t>The table that records all assets, artifacts, and project pieces that fall under the umbrella of the PHES-ODM Research Project.</t>
-  </si>
-  <si>
     <t>A tutorial video hosted on vimeo that walks users through how to use and populate the sites, polygons, and other location metadata information tables with PHES-ODM version 2.</t>
   </si>
   <si>
@@ -766,6 +756,33 @@
   </si>
   <si>
     <t>The GitHub repository for the mapping application for moving between other wastewater surveillance data structures and the ODM. It is based off an existing application called LinkML-Map, but this repository currently uses custom features in LinkML-Map that have not yet been added to a branch of the LinkML-Map repository. These new features will be added and merged soon. As such, the PHES-ODM-Mapper will not work unless you have access to these changes. Please contact mwellman@ohri.ca for questions.</t>
+  </si>
+  <si>
+    <t>odmArtifactsCSV</t>
+  </si>
+  <si>
+    <t>PHES-ODM Project Artifact List CSV version</t>
+  </si>
+  <si>
+    <t>The table that records all assets, artifacts, and project pieces that fall under the umbrella of the PHES-ODM Research Project. CSV File version.</t>
+  </si>
+  <si>
+    <t>https://github.com/PHES-ODM/.github/blob/main/Asset%20Lists%20%26%20Artifact%20Lists/artifact-list.csv</t>
+  </si>
+  <si>
+    <t>csv</t>
+  </si>
+  <si>
+    <t>odmArtifactsXLXS</t>
+  </si>
+  <si>
+    <t>PHES-ODM Project Artifact List XLSX version</t>
+  </si>
+  <si>
+    <t>The table that records all assets, artifacts, and project pieces that fall under the umbrella of the PHES-ODM Research Project. XLSX file version.</t>
+  </si>
+  <si>
+    <t>https://github.com/PHES-ODM/.github/blob/main/Asset%20Lists%20%26%20Artifact%20Lists/artifact-list.xlsx</t>
   </si>
 </sst>
 </file>
@@ -1161,7 +1178,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0B4BC87-2742-9B4D-BDFA-09F0487C7B1E}">
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.5" customWidth="1"/>
@@ -1205,7 +1222,7 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>42</v>
@@ -1231,7 +1248,7 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>43</v>
@@ -1257,7 +1274,7 @@
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>44</v>
@@ -1283,10 +1300,10 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
@@ -1309,7 +1326,7 @@
         <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>45</v>
@@ -1335,7 +1352,7 @@
         <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>46</v>
@@ -1361,7 +1378,7 @@
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>48</v>
@@ -1387,7 +1404,7 @@
         <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>49</v>
@@ -1413,7 +1430,7 @@
         <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>47</v>
@@ -1439,7 +1456,7 @@
         <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>51</v>
@@ -1465,10 +1482,10 @@
         <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="E12" t="s">
         <v>12</v>
@@ -1485,16 +1502,16 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>215</v>
+      </c>
+      <c r="B13" t="s">
+        <v>216</v>
+      </c>
+      <c r="C13" t="s">
+        <v>217</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>218</v>
-      </c>
-      <c r="B13" t="s">
-        <v>219</v>
-      </c>
-      <c r="C13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>221</v>
       </c>
       <c r="E13" t="s">
         <v>12</v>
@@ -1517,7 +1534,7 @@
         <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>53</v>
@@ -1543,7 +1560,7 @@
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>52</v>
@@ -1569,7 +1586,7 @@
         <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>41</v>
@@ -1595,7 +1612,7 @@
         <v>22</v>
       </c>
       <c r="C17" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>40</v>
@@ -1621,7 +1638,7 @@
         <v>23</v>
       </c>
       <c r="C18" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>39</v>
@@ -1647,7 +1664,7 @@
         <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>38</v>
@@ -1673,7 +1690,7 @@
         <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>37</v>
@@ -1699,7 +1716,7 @@
         <v>26</v>
       </c>
       <c r="C21" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>36</v>
@@ -1725,7 +1742,7 @@
         <v>27</v>
       </c>
       <c r="C22" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>35</v>
@@ -1751,7 +1768,7 @@
         <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>31</v>
@@ -1777,7 +1794,7 @@
         <v>29</v>
       </c>
       <c r="C24" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>30</v>
@@ -1803,7 +1820,7 @@
         <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>33</v>
@@ -1829,7 +1846,7 @@
         <v>34</v>
       </c>
       <c r="C26" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>33</v>
@@ -1855,7 +1872,7 @@
         <v>54</v>
       </c>
       <c r="C27" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>55</v>
@@ -1881,7 +1898,7 @@
         <v>56</v>
       </c>
       <c r="C28" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>57</v>
@@ -1933,7 +1950,7 @@
         <v>61</v>
       </c>
       <c r="C30" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>63</v>
@@ -1959,7 +1976,7 @@
         <v>62</v>
       </c>
       <c r="C31" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>64</v>
@@ -1985,7 +2002,7 @@
         <v>97</v>
       </c>
       <c r="C32" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>64</v>
@@ -2011,7 +2028,7 @@
         <v>65</v>
       </c>
       <c r="C33" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>66</v>
@@ -2037,7 +2054,7 @@
         <v>175</v>
       </c>
       <c r="C34" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>176</v>
@@ -2063,7 +2080,7 @@
         <v>100</v>
       </c>
       <c r="C35" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>101</v>
@@ -2089,7 +2106,7 @@
         <v>103</v>
       </c>
       <c r="C36" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>104</v>
@@ -2115,7 +2132,7 @@
         <v>110</v>
       </c>
       <c r="C37" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>106</v>
@@ -2141,7 +2158,7 @@
         <v>109</v>
       </c>
       <c r="C38" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>117</v>
@@ -2167,7 +2184,7 @@
         <v>118</v>
       </c>
       <c r="C39" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>114</v>
@@ -2193,7 +2210,7 @@
         <v>119</v>
       </c>
       <c r="C40" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>115</v>
@@ -2219,7 +2236,7 @@
         <v>120</v>
       </c>
       <c r="C41" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>116</v>
@@ -2245,7 +2262,7 @@
         <v>121</v>
       </c>
       <c r="C42" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>122</v>
@@ -2271,7 +2288,7 @@
         <v>124</v>
       </c>
       <c r="C43" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>123</v>
@@ -2297,7 +2314,7 @@
         <v>125</v>
       </c>
       <c r="C44" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>126</v>
@@ -2323,7 +2340,7 @@
         <v>127</v>
       </c>
       <c r="C45" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>128</v>
@@ -2349,7 +2366,7 @@
         <v>129</v>
       </c>
       <c r="C46" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>130</v>
@@ -2375,7 +2392,7 @@
         <v>137</v>
       </c>
       <c r="C47" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>138</v>
@@ -2401,7 +2418,7 @@
         <v>139</v>
       </c>
       <c r="C48" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>140</v>
@@ -2453,7 +2470,7 @@
         <v>147</v>
       </c>
       <c r="C50" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>148</v>
@@ -2479,7 +2496,7 @@
         <v>150</v>
       </c>
       <c r="C51" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>149</v>
@@ -2505,7 +2522,7 @@
         <v>153</v>
       </c>
       <c r="C52" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>152</v>
@@ -2531,7 +2548,7 @@
         <v>156</v>
       </c>
       <c r="C53" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>155</v>
@@ -2557,7 +2574,7 @@
         <v>161</v>
       </c>
       <c r="C54" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>158</v>
@@ -2583,7 +2600,7 @@
         <v>160</v>
       </c>
       <c r="C55" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>159</v>
@@ -2609,7 +2626,7 @@
         <v>163</v>
       </c>
       <c r="C56" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>162</v>
@@ -2635,7 +2652,7 @@
         <v>164</v>
       </c>
       <c r="C57" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>165</v>
@@ -2655,24 +2672,53 @@
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>181</v>
+        <v>240</v>
       </c>
       <c r="B58" t="s">
+        <v>241</v>
+      </c>
+      <c r="C58" t="s">
+        <v>242</v>
+      </c>
+      <c r="D58" t="s">
+        <v>243</v>
+      </c>
+      <c r="E58" t="s">
+        <v>12</v>
+      </c>
+      <c r="F58" t="s">
+        <v>244</v>
+      </c>
+      <c r="G58" t="s">
+        <v>179</v>
+      </c>
+      <c r="H58" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>245</v>
+      </c>
+      <c r="B59" t="s">
+        <v>246</v>
+      </c>
+      <c r="C59" t="s">
+        <v>247</v>
+      </c>
+      <c r="D59" t="s">
+        <v>248</v>
+      </c>
+      <c r="E59" t="s">
+        <v>12</v>
+      </c>
+      <c r="F59" t="s">
         <v>180</v>
       </c>
-      <c r="C58" t="s">
-        <v>183</v>
-      </c>
-      <c r="E58" t="s">
-        <v>12</v>
-      </c>
-      <c r="F58" t="s">
-        <v>182</v>
-      </c>
-      <c r="G58" t="s">
-        <v>179</v>
-      </c>
-      <c r="H58" t="s">
+      <c r="G59" t="s">
+        <v>179</v>
+      </c>
+      <c r="H59" t="s">
         <v>170</v>
       </c>
     </row>

</xml_diff>